<commit_message>
#15 - déplacement du numero AMC en tant que identifier de Organization + MAJ des exemples + MAJ du narratif ccffde4a3e09e0932d26f5d27a96deec4b476353
</commit_message>
<xml_diff>
--- a/nmoreau/ig/StructureDefinition-fr-coverage-amc-extended.xlsx
+++ b/nmoreau/ig/StructureDefinition-fr-coverage-amc-extended.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AK$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AK$21</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1049" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="135">
   <si>
     <t>Property</t>
   </si>
@@ -45,7 +45,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Extension AMC Étendue</t>
+    <t>Extension AMC Étendue ROC</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-22T09:09:51+00:00</t>
+    <t>2025-10-28T10:00:18+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -295,11 +295,21 @@
     <t>Extension.extension</t>
   </si>
   <si>
+    <t>extensions
+user content</t>
+  </si>
+  <si>
     <t xml:space="preserve">Extension
 </t>
   </si>
   <si>
-    <t>An Extension</t>
+    <t>Additional content defined by implementations</t>
+  </si>
+  <si>
+    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
+  </si>
+  <si>
+    <t>There can be no stigma associated with the use of extensions by any application, project, or standard - regardless of the institution or jurisdiction that uses or defines the extensions.  The use of extensions is what allows the FHIR specification to retain a core level of simplicity for everyone.</t>
   </si>
   <si>
     <t xml:space="preserve">value:url}
@@ -315,28 +325,31 @@
     <t>Element.extension</t>
   </si>
   <si>
-    <t>Extension.extension:nomAMC</t>
-  </si>
-  <si>
-    <t>nomAMC</t>
+    <t>Extension.extension:codeConvention</t>
+  </si>
+  <si>
+    <t>codeConvention</t>
   </si>
   <si>
     <t>Y</t>
   </si>
   <si>
-    <t>Extension.extension:nomAMC.id</t>
+    <t>An Extension</t>
+  </si>
+  <si>
+    <t>Extension.extension:codeConvention.id</t>
   </si>
   <si>
     <t>Extension.extension.id</t>
   </si>
   <si>
-    <t>Extension.extension:nomAMC.extension</t>
+    <t>Extension.extension:codeConvention.extension</t>
   </si>
   <si>
     <t>Extension.extension.extension</t>
   </si>
   <si>
-    <t>Extension.extension:nomAMC.url</t>
+    <t>Extension.extension:codeConvention.url</t>
   </si>
   <si>
     <t>Extension.extension.url</t>
@@ -361,7 +374,7 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>Extension.extension:nomAMC.value[x]</t>
+    <t>Extension.extension:codeConvention.value[x]</t>
   </si>
   <si>
     <t>Extension.extension.value[x]</t>
@@ -378,42 +391,6 @@
   <si>
     <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
 </t>
-  </si>
-  <si>
-    <t>Extension.extension:numeroAMC</t>
-  </si>
-  <si>
-    <t>numeroAMC</t>
-  </si>
-  <si>
-    <t>Extension.extension:numeroAMC.id</t>
-  </si>
-  <si>
-    <t>Extension.extension:numeroAMC.extension</t>
-  </si>
-  <si>
-    <t>Extension.extension:numeroAMC.url</t>
-  </si>
-  <si>
-    <t>Extension.extension:numeroAMC.value[x]</t>
-  </si>
-  <si>
-    <t>Extension.extension:codeConvention</t>
-  </si>
-  <si>
-    <t>codeConvention</t>
-  </si>
-  <si>
-    <t>Extension.extension:codeConvention.id</t>
-  </si>
-  <si>
-    <t>Extension.extension:codeConvention.extension</t>
-  </si>
-  <si>
-    <t>Extension.extension:codeConvention.url</t>
-  </si>
-  <si>
-    <t>Extension.extension:codeConvention.value[x]</t>
   </si>
   <si>
     <t>Extension.extension:codeCSR</t>
@@ -786,13 +763,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK31"/>
+  <dimension ref="A1:AK21"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="38.26953125" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="24.9921875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="13.64453125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="7.6796875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="10.83984375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="4.65625" customWidth="true" bestFit="true"/>
@@ -1155,11 +1132,11 @@
       </c>
       <c r="C4" s="2"/>
       <c r="D4" t="s" s="2">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" t="s" s="2">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="G4" t="s" s="2">
         <v>79</v>
@@ -1174,15 +1151,17 @@
         <v>77</v>
       </c>
       <c r="K4" t="s" s="2">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L4" t="s" s="2">
-        <v>31</v>
+        <v>93</v>
       </c>
       <c r="M4" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="N4" s="2"/>
+        <v>94</v>
+      </c>
+      <c r="N4" t="s" s="2">
+        <v>95</v>
+      </c>
       <c r="O4" s="2"/>
       <c r="P4" t="s" s="2">
         <v>77</v>
@@ -1219,19 +1198,19 @@
         <v>77</v>
       </c>
       <c r="AB4" t="s" s="2">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="AC4" t="s" s="2">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="AD4" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE4" t="s" s="2">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AF4" t="s" s="2">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AG4" t="s" s="2">
         <v>78</v>
@@ -1246,18 +1225,18 @@
         <v>82</v>
       </c>
       <c r="AK4" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" hidden="true">
       <c r="A5" t="s" s="2">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B5" t="s" s="2">
         <v>90</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D5" t="s" s="2">
         <v>77</v>
@@ -1270,7 +1249,7 @@
         <v>84</v>
       </c>
       <c r="H5" t="s" s="2">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="I5" t="s" s="2">
         <v>77</v>
@@ -1279,13 +1258,13 @@
         <v>77</v>
       </c>
       <c r="K5" t="s" s="2">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L5" t="s" s="2">
         <v>31</v>
       </c>
       <c r="M5" t="s" s="2">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -1336,7 +1315,7 @@
         <v>77</v>
       </c>
       <c r="AF5" t="s" s="2">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AG5" t="s" s="2">
         <v>78</v>
@@ -1356,10 +1335,10 @@
     </row>
     <row r="6" hidden="true">
       <c r="A6" t="s" s="2">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
@@ -1459,10 +1438,10 @@
     </row>
     <row r="7" hidden="true">
       <c r="A7" t="s" s="2">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
@@ -1485,13 +1464,13 @@
         <v>77</v>
       </c>
       <c r="K7" t="s" s="2">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L7" t="s" s="2">
         <v>31</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1530,19 +1509,19 @@
         <v>77</v>
       </c>
       <c r="AB7" t="s" s="2">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="AC7" t="s" s="2">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="AD7" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE7" t="s" s="2">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>78</v>
@@ -1562,10 +1541,10 @@
     </row>
     <row r="8" hidden="true">
       <c r="A8" t="s" s="2">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1588,16 +1567,16 @@
         <v>77</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="N8" t="s" s="2">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" t="s" s="2">
@@ -1605,7 +1584,7 @@
       </c>
       <c r="Q8" s="2"/>
       <c r="R8" t="s" s="2">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="S8" t="s" s="2">
         <v>77</v>
@@ -1647,7 +1626,7 @@
         <v>77</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>84</v>
@@ -1662,15 +1641,15 @@
         <v>77</v>
       </c>
       <c r="AK8" t="s" s="2">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" hidden="true">
       <c r="A9" t="s" s="2">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -1696,10 +1675,10 @@
         <v>85</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -1750,7 +1729,7 @@
         <v>77</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>78</v>
@@ -1762,34 +1741,34 @@
         <v>77</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="AK9" t="s" s="2">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" hidden="true">
       <c r="A10" t="s" s="2">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B10" t="s" s="2">
         <v>90</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D10" t="s" s="2">
         <v>77</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" t="s" s="2">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="G10" t="s" s="2">
         <v>84</v>
       </c>
       <c r="H10" t="s" s="2">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="I10" t="s" s="2">
         <v>77</v>
@@ -1798,13 +1777,13 @@
         <v>77</v>
       </c>
       <c r="K10" t="s" s="2">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L10" t="s" s="2">
         <v>31</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -1855,7 +1834,7 @@
         <v>77</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>78</v>
@@ -1875,10 +1854,10 @@
     </row>
     <row r="11" hidden="true">
       <c r="A11" t="s" s="2">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -1978,10 +1957,10 @@
     </row>
     <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2004,13 +1983,13 @@
         <v>77</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L12" t="s" s="2">
         <v>31</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -2049,19 +2028,19 @@
         <v>77</v>
       </c>
       <c r="AB12" t="s" s="2">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="AC12" t="s" s="2">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="AD12" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE12" t="s" s="2">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>78</v>
@@ -2081,10 +2060,10 @@
     </row>
     <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2107,16 +2086,16 @@
         <v>77</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -2124,7 +2103,7 @@
       </c>
       <c r="Q13" s="2"/>
       <c r="R13" t="s" s="2">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="S13" t="s" s="2">
         <v>77</v>
@@ -2166,7 +2145,7 @@
         <v>77</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>84</v>
@@ -2181,15 +2160,15 @@
         <v>77</v>
       </c>
       <c r="AK13" t="s" s="2">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2215,10 +2194,10 @@
         <v>85</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2269,7 +2248,7 @@
         <v>77</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>78</v>
@@ -2281,21 +2260,21 @@
         <v>77</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="AK14" t="s" s="2">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B15" t="s" s="2">
         <v>90</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D15" t="s" s="2">
         <v>77</v>
@@ -2308,7 +2287,7 @@
         <v>84</v>
       </c>
       <c r="H15" t="s" s="2">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="I15" t="s" s="2">
         <v>77</v>
@@ -2317,13 +2296,13 @@
         <v>77</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L15" t="s" s="2">
         <v>31</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2374,7 +2353,7 @@
         <v>77</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>78</v>
@@ -2394,10 +2373,10 @@
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2497,10 +2476,10 @@
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -2523,13 +2502,13 @@
         <v>77</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L17" t="s" s="2">
         <v>31</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -2568,19 +2547,19 @@
         <v>77</v>
       </c>
       <c r="AB17" t="s" s="2">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="AC17" t="s" s="2">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="AD17" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE17" t="s" s="2">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>78</v>
@@ -2600,10 +2579,10 @@
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -2626,16 +2605,16 @@
         <v>77</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="N18" t="s" s="2">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -2643,7 +2622,7 @@
       </c>
       <c r="Q18" s="2"/>
       <c r="R18" t="s" s="2">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="S18" t="s" s="2">
         <v>77</v>
@@ -2685,7 +2664,7 @@
         <v>77</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>84</v>
@@ -2700,15 +2679,15 @@
         <v>77</v>
       </c>
       <c r="AK18" t="s" s="2">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -2734,10 +2713,10 @@
         <v>85</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -2788,7 +2767,7 @@
         <v>77</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>78</v>
@@ -2800,34 +2779,32 @@
         <v>77</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="C20" t="s" s="2">
-        <v>131</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
         <v>77</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="G20" t="s" s="2">
         <v>84</v>
       </c>
       <c r="H20" t="s" s="2">
-        <v>99</v>
+        <v>77</v>
       </c>
       <c r="I20" t="s" s="2">
         <v>77</v>
@@ -2836,22 +2813,24 @@
         <v>77</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>31</v>
+        <v>111</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="N20" s="2"/>
+        <v>112</v>
+      </c>
+      <c r="N20" t="s" s="2">
+        <v>113</v>
+      </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
         <v>77</v>
       </c>
       <c r="Q20" s="2"/>
       <c r="R20" t="s" s="2">
-        <v>77</v>
+        <v>3</v>
       </c>
       <c r="S20" t="s" s="2">
         <v>77</v>
@@ -2893,30 +2872,30 @@
         <v>77</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="AG20" t="s" s="2">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="AH20" t="s" s="2">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="AI20" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>77</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -2927,7 +2906,7 @@
         <v>78</v>
       </c>
       <c r="G21" t="s" s="2">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="H21" t="s" s="2">
         <v>77</v>
@@ -2939,13 +2918,13 @@
         <v>77</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>85</v>
+        <v>134</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>86</v>
+        <v>118</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>87</v>
+        <v>119</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -2996,7 +2975,7 @@
         <v>77</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>88</v>
+        <v>120</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>78</v>
@@ -3008,1052 +2987,14 @@
         <v>77</v>
       </c>
       <c r="AJ21" t="s" s="2">
-        <v>77</v>
+        <v>121</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="22" hidden="true">
-      <c r="A22" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="B22" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="C22" s="2"/>
-      <c r="D22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E22" s="2"/>
-      <c r="F22" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G22" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="H22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K22" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="L22" t="s" s="2">
-        <v>31</v>
-      </c>
-      <c r="M22" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
-      <c r="P22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q22" s="2"/>
-      <c r="R22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB22" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AC22" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="AD22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE22" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="AF22" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AG22" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH22" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI22" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ22" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK22" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="23" hidden="true">
-      <c r="A23" t="s" s="2">
-        <v>134</v>
-      </c>
-      <c r="B23" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="C23" s="2"/>
-      <c r="D23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E23" s="2"/>
-      <c r="F23" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="G23" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K23" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="L23" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="M23" t="s" s="2">
-        <v>108</v>
-      </c>
-      <c r="N23" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="O23" s="2"/>
-      <c r="P23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q23" s="2"/>
-      <c r="R23" t="s" s="2">
-        <v>131</v>
-      </c>
-      <c r="S23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF23" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="AG23" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH23" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ23" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AK23" t="s" s="2">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="24" hidden="true">
-      <c r="A24" t="s" s="2">
-        <v>135</v>
-      </c>
-      <c r="B24" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="C24" s="2"/>
-      <c r="D24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E24" s="2"/>
-      <c r="F24" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G24" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K24" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="L24" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="M24" t="s" s="2">
         <v>115</v>
       </c>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
-      <c r="P24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q24" s="2"/>
-      <c r="R24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF24" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="AG24" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH24" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ24" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="AK24" t="s" s="2">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="25" hidden="true">
-      <c r="A25" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="B25" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="C25" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="D25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E25" s="2"/>
-      <c r="F25" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G25" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H25" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="I25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K25" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="L25" t="s" s="2">
-        <v>31</v>
-      </c>
-      <c r="M25" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
-      <c r="P25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q25" s="2"/>
-      <c r="R25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF25" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AG25" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH25" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI25" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ25" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK25" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="26" hidden="true">
-      <c r="A26" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="B26" t="s" s="2">
-        <v>101</v>
-      </c>
-      <c r="C26" s="2"/>
-      <c r="D26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E26" s="2"/>
-      <c r="F26" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G26" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K26" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="L26" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="M26" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
-      <c r="P26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q26" s="2"/>
-      <c r="R26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF26" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AG26" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH26" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AK26" t="s" s="2">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="27" hidden="true">
-      <c r="A27" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="B27" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="C27" s="2"/>
-      <c r="D27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E27" s="2"/>
-      <c r="F27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="H27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K27" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="L27" t="s" s="2">
-        <v>31</v>
-      </c>
-      <c r="M27" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="N27" s="2"/>
-      <c r="O27" s="2"/>
-      <c r="P27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q27" s="2"/>
-      <c r="R27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB27" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AC27" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="AD27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE27" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="AF27" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AG27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH27" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ27" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK27" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="28" hidden="true">
-      <c r="A28" t="s" s="2">
-        <v>140</v>
-      </c>
-      <c r="B28" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="C28" s="2"/>
-      <c r="D28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E28" s="2"/>
-      <c r="F28" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="G28" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K28" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="L28" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="M28" t="s" s="2">
-        <v>108</v>
-      </c>
-      <c r="N28" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="O28" s="2"/>
-      <c r="P28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q28" s="2"/>
-      <c r="R28" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="S28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF28" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="AG28" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH28" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AK28" t="s" s="2">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="29" hidden="true">
-      <c r="A29" t="s" s="2">
-        <v>141</v>
-      </c>
-      <c r="B29" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="C29" s="2"/>
-      <c r="D29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E29" s="2"/>
-      <c r="F29" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G29" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K29" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="L29" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="M29" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="N29" s="2"/>
-      <c r="O29" s="2"/>
-      <c r="P29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q29" s="2"/>
-      <c r="R29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF29" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="AG29" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH29" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ29" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="AK29" t="s" s="2">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="30" hidden="true">
-      <c r="A30" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="B30" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E30" s="2"/>
-      <c r="F30" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="G30" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K30" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="L30" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="M30" t="s" s="2">
-        <v>108</v>
-      </c>
-      <c r="N30" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="O30" s="2"/>
-      <c r="P30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q30" s="2"/>
-      <c r="R30" t="s" s="2">
-        <v>3</v>
-      </c>
-      <c r="S30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF30" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="AG30" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH30" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AK30" t="s" s="2">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="31" hidden="true">
-      <c r="A31" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="B31" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="C31" s="2"/>
-      <c r="D31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E31" s="2"/>
-      <c r="F31" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G31" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="H31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K31" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="L31" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="M31" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2"/>
-      <c r="P31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q31" s="2"/>
-      <c r="R31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF31" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="AG31" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH31" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ31" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="AK31" t="s" s="2">
-        <v>111</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AK31">
+  <autoFilter ref="A1:AK21">
     <filterColumn colId="6">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -4063,7 +3004,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI30">
+  <conditionalFormatting sqref="A2:AI20">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>